<commit_message>
NWSS to ODM v2 ID code updates
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/nwss-reporting-to-v2/ids/nwss_reporting_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/nwss-reporting-to-v2/ids/nwss_reporting_to_v2_id_code.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/nwss-reporting-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E627A01F-9A80-0B4B-9AC2-DB2FC522D8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0DBE58-EEC1-A04B-97E8-92AD6BD097ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="15940" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
   <sheets>
-    <sheet name="sites" sheetId="1" r:id="rId1"/>
+    <sheet name="id_code" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
Removed all ID generation code for NWSS (does not need to override the general ID code)
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/nwss-reporting-to-v2/ids/nwss_reporting_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/nwss-reporting-to-v2/ids/nwss_reporting_to_v2_id_code.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/nwss-reporting-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0DBE58-EEC1-A04B-97E8-92AD6BD097ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48727D48-FC18-904B-9215-F23680DE0BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="15940" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
   <sheets>
     <sheet name="id_code" sheetId="1" r:id="rId1"/>
@@ -35,10 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
-  <si>
-    <t>sites</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>class</t>
   </si>
@@ -47,36 +44,6 @@
   </si>
   <si>
     <t>code0</t>
-  </si>
-  <si>
-    <t>sampleShed</t>
-  </si>
-  <si>
-    <t>def get_sample_shed_type(check_first, check_with_prefix, prefix):
-    if check_first is not None and len(str(check_first)) &gt; 0:
-        if not isinstance(check_first, list):
-            check_first = [check_first]
-        for cur in check_first:
-            if cur and len(cur) &gt; 0:
-                return cur
-    for val in check_with_prefix:
-        if str(val).startswith(prefix):
-            return str(val).split(prefix, maxsplit=1)[1]
-    return ''        
-#target = get_sample_shed_type(dat.sites.__siteType, dat.sites.__sampleShed, 'siteType:')
-target = get_sample_shed_type(None, dat.sites.__sampleShed, 'sampleShed:')</t>
-  </si>
-  <si>
-    <t>""</t>
-  </si>
-  <si>
-    <t>qualityReports</t>
-  </si>
-  <si>
-    <t>measureRepID</t>
-  </si>
-  <si>
-    <t>sampleID</t>
   </si>
 </sst>
 </file>
@@ -120,12 +87,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -144,9 +108,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -184,7 +148,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -290,7 +254,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -432,7 +396,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -440,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB192A8-54D6-B94E-B895-8C1E220F8CDD}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -450,48 +414,15 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4" ht="356" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Linking of protocolRelationships.stepIDObj, stepIDSub, and protocolIDContainer
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/nwss-reporting-to-v2/ids/nwss_reporting_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/nwss-reporting-to-v2/ids/nwss_reporting_to_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/nwss-reporting-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48727D48-FC18-904B-9215-F23680DE0BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB5C094-591E-6441-9DF9-9AFB1124DE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>class</t>
   </si>
@@ -44,6 +44,27 @@
   </si>
   <si>
     <t>code0</t>
+  </si>
+  <si>
+    <t>protocolRelationships</t>
+  </si>
+  <si>
+    <t>stepIDObj</t>
+  </si>
+  <si>
+    <t>stepIDSub</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_subject")</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_object")</t>
+  </si>
+  <si>
+    <t>dat.protocols.protocolID</t>
+  </si>
+  <si>
+    <t>protocolIDContainer</t>
   </si>
 </sst>
 </file>
@@ -404,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB192A8-54D6-B94E-B895-8C1E220F8CDD}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -424,6 +445,39 @@
       </c>
       <c r="D1" s="1"/>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>